<commit_message>
chore(mappa): aggiornamento automatico 2026-08-31
</commit_message>
<xml_diff>
--- a/Torino_2027.xlsx
+++ b/Torino_2027.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scarg\Dropbox\PNE Simone\Guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0933A056-CA54-427D-9894-CF5803C0F911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA60B790-70E9-4F01-B69B-847B14EF757C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="665" xr2:uid="{65E54767-2A5A-433C-9949-276C98563996}"/>
   </bookViews>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="917">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2020" uniqueCount="916">
   <si>
     <t>Recensore</t>
   </si>
@@ -1811,9 +1811,6 @@
   </si>
   <si>
     <t>1 nuvola, 1 focaccia o pizza crunch, 1 pizza contemporanea</t>
-  </si>
-  <si>
-    <t>33</t>
   </si>
   <si>
     <t>Tartatea Torteria</t>
@@ -3725,15 +3722,15 @@
       </c>
       <c r="F4" s="10">
         <f>+AE6</f>
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G4" s="10">
         <f>+AG6</f>
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H4" s="7">
         <f>+E4-G4</f>
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I4" s="21" t="s">
         <v>16</v>
@@ -3755,18 +3752,18 @@
       </c>
       <c r="F5" s="12">
         <f>+F3+F4</f>
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G5" s="12">
         <f>+G3+G4</f>
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H5" s="12">
         <f>+H3+H4</f>
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I5" s="22" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="J5" s="13"/>
       <c r="K5" s="13"/>
@@ -3856,7 +3853,7 @@
       </c>
       <c r="AE6" s="2">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="AF6" s="2">
         <f t="shared" si="1"/>
@@ -3864,7 +3861,7 @@
       </c>
       <c r="AG6" s="2">
         <f t="shared" si="1"/>
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="AH6" s="2">
         <f t="shared" si="1"/>
@@ -3877,13 +3874,13 @@
     </row>
     <row r="7" spans="1:46" s="26" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
+        <v>681</v>
+      </c>
+      <c r="B7" s="23" t="s">
         <v>682</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="C7" s="23" t="s">
         <v>683</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>684</v>
       </c>
       <c r="D7" s="27" t="s">
         <v>13</v>
@@ -3904,16 +3901,16 @@
         <v>11</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="K7" s="29" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="L7" s="23" t="s">
         <v>19</v>
       </c>
       <c r="M7" s="27" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="N7" s="24" t="s">
         <v>0</v>
@@ -3925,7 +3922,7 @@
         <v>2</v>
       </c>
       <c r="Q7" s="42" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="R7" s="25"/>
       <c r="S7" s="25">
@@ -4009,22 +4006,22 @@
         <v>1</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E8" s="34" t="s">
         <v>236</v>
       </c>
       <c r="F8" s="34" t="s">
+        <v>658</v>
+      </c>
+      <c r="G8" s="34" t="s">
         <v>659</v>
-      </c>
-      <c r="G8" s="34" t="s">
-        <v>660</v>
       </c>
       <c r="H8" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I8" s="33" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J8" s="33">
         <v>99</v>
@@ -4033,13 +4030,13 @@
         <v>300</v>
       </c>
       <c r="L8" s="33" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="M8" s="34" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="N8" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O8" s="35">
         <v>1</v>
@@ -4165,7 +4162,7 @@
         <v>103</v>
       </c>
       <c r="N9" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O9" s="35">
         <v>1</v>
@@ -4290,10 +4287,10 @@
         <v>130</v>
       </c>
       <c r="M10" s="34" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="N10" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O10" s="35">
         <v>1</v>
@@ -4395,7 +4392,7 @@
         <v>236</v>
       </c>
       <c r="F11" s="34" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="G11" s="34" t="s">
         <v>107</v>
@@ -4410,16 +4407,16 @@
         <v>99</v>
       </c>
       <c r="K11" s="33" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="L11" s="33" t="s">
+        <v>679</v>
+      </c>
+      <c r="M11" s="34" t="s">
         <v>680</v>
       </c>
-      <c r="M11" s="34" t="s">
-        <v>681</v>
-      </c>
       <c r="N11" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O11" s="35">
         <v>1</v>
@@ -4515,13 +4512,13 @@
         <v>1</v>
       </c>
       <c r="D12" s="40" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E12" s="40" t="s">
         <v>278</v>
       </c>
       <c r="F12" s="40" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="G12" s="40" t="s">
         <v>371</v>
@@ -4530,7 +4527,7 @@
         <v>190</v>
       </c>
       <c r="I12" s="39" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="J12" s="39">
         <v>99</v>
@@ -4539,10 +4536,10 @@
         <v>300</v>
       </c>
       <c r="L12" s="39" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="M12" s="40" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="N12" s="40"/>
       <c r="O12" s="41"/>
@@ -4667,7 +4664,7 @@
         <v>103</v>
       </c>
       <c r="N13" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O13" s="35">
         <v>1</v>
@@ -4765,13 +4762,13 @@
         <v>1</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E14" s="37" t="s">
         <v>278</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="G14" s="37" t="s">
         <v>88</v>
@@ -4780,7 +4777,7 @@
         <v>190</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="J14" s="36">
         <v>2</v>
@@ -4795,7 +4792,7 @@
         <v>195</v>
       </c>
       <c r="N14" s="37" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O14" s="38"/>
       <c r="P14" s="36"/>
@@ -4889,20 +4886,20 @@
         <v>2</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="E15" s="31" t="s">
         <v>278</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="G15" s="31"/>
       <c r="H15" s="31" t="s">
         <v>190</v>
       </c>
       <c r="I15" s="30" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="J15" s="30"/>
       <c r="K15" s="30" t="s">
@@ -5005,13 +5002,13 @@
         <v>2</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="G16" s="19" t="s">
         <v>82</v>
@@ -5020,7 +5017,7 @@
         <v>190</v>
       </c>
       <c r="I16" s="20" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="J16" s="20">
         <v>1</v>
@@ -5127,22 +5124,22 @@
         <v>2</v>
       </c>
       <c r="D17" s="34" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E17" s="34" t="s">
         <v>235</v>
       </c>
       <c r="F17" s="34" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="G17" s="34" t="s">
         <v>103</v>
       </c>
       <c r="H17" s="34" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="J17" s="33">
         <v>99</v>
@@ -5154,10 +5151,10 @@
         <v>47</v>
       </c>
       <c r="M17" s="34" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="N17" s="34" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="O17" s="35">
         <v>1</v>
@@ -5253,22 +5250,22 @@
         <v>2</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="E18" s="37" t="s">
         <v>235</v>
       </c>
       <c r="F18" s="37" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="G18" s="37" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="H18" s="37" t="s">
         <v>190</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="J18" s="36"/>
       <c r="K18" s="36" t="s">
@@ -5278,10 +5275,10 @@
         <v>45</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="N18" s="37" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O18" s="38"/>
       <c r="P18" s="36"/>
@@ -5524,10 +5521,10 @@
         <v>507</v>
       </c>
       <c r="M20" s="34" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="N20" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O20" s="35">
         <v>1</v>
@@ -5774,10 +5771,10 @@
         <v>301</v>
       </c>
       <c r="M22" s="34" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="N22" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O22" s="35">
         <v>1</v>
@@ -5905,7 +5902,7 @@
         <v>246</v>
       </c>
       <c r="N23" s="34" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O23" s="35">
         <v>1</v>
@@ -6031,7 +6028,7 @@
         <v>510</v>
       </c>
       <c r="N24" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O24" s="35">
         <v>1</v>
@@ -6127,22 +6124,22 @@
         <v>2</v>
       </c>
       <c r="D25" s="34" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="E25" s="34" t="s">
         <v>278</v>
       </c>
       <c r="F25" s="34" t="s">
+        <v>598</v>
+      </c>
+      <c r="G25" s="34" t="s">
         <v>599</v>
-      </c>
-      <c r="G25" s="34" t="s">
-        <v>600</v>
       </c>
       <c r="H25" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I25" s="33" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="J25" s="33">
         <v>99</v>
@@ -6151,13 +6148,13 @@
         <v>290</v>
       </c>
       <c r="L25" s="33" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="M25" s="34" t="s">
         <v>195</v>
       </c>
       <c r="N25" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O25" s="35">
         <v>1</v>
@@ -6259,10 +6256,10 @@
         <v>235</v>
       </c>
       <c r="F26" s="34" t="s">
+        <v>764</v>
+      </c>
+      <c r="G26" s="34" t="s">
         <v>765</v>
-      </c>
-      <c r="G26" s="34" t="s">
-        <v>766</v>
       </c>
       <c r="H26" s="34" t="s">
         <v>190</v>
@@ -6283,7 +6280,7 @@
         <v>195</v>
       </c>
       <c r="N26" s="34" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O26" s="35">
         <v>1</v>
@@ -6409,7 +6406,7 @@
         <v>103</v>
       </c>
       <c r="N27" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O27" s="35">
         <v>1</v>
@@ -6507,13 +6504,13 @@
         <v>2</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>236</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="G28" s="19" t="s">
         <v>137</v>
@@ -6522,7 +6519,7 @@
         <v>190</v>
       </c>
       <c r="I28" s="20" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="J28" s="20">
         <v>6</v>
@@ -6531,7 +6528,7 @@
         <v>385</v>
       </c>
       <c r="L28" s="20" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="M28" s="19" t="s">
         <v>195</v>
@@ -6629,13 +6626,13 @@
         <v>2</v>
       </c>
       <c r="D29" s="34" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="E29" s="34" t="s">
         <v>278</v>
       </c>
       <c r="F29" s="34" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="G29" s="34" t="s">
         <v>88</v>
@@ -6644,7 +6641,7 @@
         <v>190</v>
       </c>
       <c r="I29" s="33" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="J29" s="33">
         <v>2</v>
@@ -6656,10 +6653,10 @@
         <v>507</v>
       </c>
       <c r="M29" s="34" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="N29" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O29" s="35">
         <v>1</v>
@@ -6780,10 +6777,10 @@
       </c>
       <c r="L30" s="36"/>
       <c r="M30" s="37" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="N30" s="37" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O30" s="38"/>
       <c r="P30" s="36"/>
@@ -6901,18 +6898,18 @@
         <v>300</v>
       </c>
       <c r="L31" s="36" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="M31" s="37" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="N31" s="37" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O31" s="38"/>
       <c r="P31" s="36"/>
       <c r="Q31" s="37" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="R31" s="13"/>
       <c r="S31" s="2">
@@ -7033,7 +7030,7 @@
         <v>246</v>
       </c>
       <c r="N32" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O32" s="35">
         <v>1</v>
@@ -7129,11 +7126,11 @@
         <v>2</v>
       </c>
       <c r="D33" s="34" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="E33" s="34"/>
       <c r="F33" s="34" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="G33" s="34" t="s">
         <v>88</v>
@@ -7142,7 +7139,7 @@
         <v>190</v>
       </c>
       <c r="I33" s="33" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="J33" s="33"/>
       <c r="K33" s="33" t="s">
@@ -7151,7 +7148,7 @@
       <c r="L33" s="33"/>
       <c r="M33" s="34"/>
       <c r="N33" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O33" s="35">
         <v>1</v>
@@ -7249,13 +7246,13 @@
         <v>2</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="E34" s="19" t="s">
         <v>278</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="G34" s="19" t="s">
         <v>82</v>
@@ -7264,7 +7261,7 @@
         <v>190</v>
       </c>
       <c r="I34" s="20" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="J34" s="20"/>
       <c r="K34" s="20" t="s">
@@ -7274,7 +7271,7 @@
         <v>75</v>
       </c>
       <c r="M34" s="19" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="N34" s="19"/>
       <c r="O34" s="18"/>
@@ -7396,7 +7393,7 @@
         <v>505</v>
       </c>
       <c r="M35" s="19" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="N35" s="19"/>
       <c r="O35" s="18"/>
@@ -7491,22 +7488,22 @@
         <v>3</v>
       </c>
       <c r="D36" s="34" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="E36" s="34" t="s">
         <v>234</v>
       </c>
       <c r="F36" s="34" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="G36" s="34" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="H36" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I36" s="33" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="J36" s="33"/>
       <c r="K36" s="33" t="s">
@@ -7516,17 +7513,17 @@
         <v>55</v>
       </c>
       <c r="M36" s="34" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="N36" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O36" s="35">
         <v>1</v>
       </c>
       <c r="P36" s="33"/>
       <c r="Q36" s="34" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="R36" s="13"/>
       <c r="S36" s="2">
@@ -7647,7 +7644,7 @@
         <v>195</v>
       </c>
       <c r="N37" s="37" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="O37" s="38"/>
       <c r="P37" s="36"/>
@@ -7771,7 +7768,7 @@
         <v>304</v>
       </c>
       <c r="N38" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O38" s="35">
         <v>1</v>
@@ -7869,22 +7866,22 @@
         <v>3</v>
       </c>
       <c r="D39" s="37" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="E39" s="37" t="s">
         <v>234</v>
       </c>
       <c r="F39" s="37" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="G39" s="37" t="s">
         <v>103</v>
       </c>
       <c r="H39" s="37" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="I39" s="36" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="J39" s="36">
         <v>99</v>
@@ -7896,10 +7893,10 @@
         <v>65</v>
       </c>
       <c r="M39" s="37" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="N39" s="37" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O39" s="38"/>
       <c r="P39" s="36"/>
@@ -8008,7 +8005,7 @@
         <v>190</v>
       </c>
       <c r="I40" s="20" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="J40" s="20">
         <v>99</v>
@@ -8020,7 +8017,7 @@
         <v>305</v>
       </c>
       <c r="M40" s="19" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="N40" s="19"/>
       <c r="O40" s="18"/>
@@ -8115,13 +8112,13 @@
         <v>3</v>
       </c>
       <c r="D41" s="37" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="E41" s="37" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="F41" s="37" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="G41" s="37" t="s">
         <v>82</v>
@@ -8130,7 +8127,7 @@
         <v>190</v>
       </c>
       <c r="I41" s="36" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="J41" s="36">
         <v>1</v>
@@ -8142,10 +8139,10 @@
         <v>50</v>
       </c>
       <c r="M41" s="37" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="N41" s="37" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O41" s="38"/>
       <c r="P41" s="36"/>
@@ -8239,13 +8236,13 @@
         <v>3</v>
       </c>
       <c r="D42" s="34" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="E42" s="34" t="s">
         <v>234</v>
       </c>
       <c r="F42" s="34" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="G42" s="34" t="s">
         <v>102</v>
@@ -8254,7 +8251,7 @@
         <v>190</v>
       </c>
       <c r="I42" s="33" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="J42" s="33">
         <v>2</v>
@@ -8266,10 +8263,10 @@
         <v>505</v>
       </c>
       <c r="M42" s="34" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="N42" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O42" s="35">
         <v>1</v>
@@ -8392,7 +8389,7 @@
         <v>40</v>
       </c>
       <c r="M43" s="19" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="N43" s="19"/>
       <c r="O43" s="18"/>
@@ -8636,7 +8633,7 @@
         <v>38</v>
       </c>
       <c r="M45" s="19" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="N45" s="19"/>
       <c r="O45" s="18"/>
@@ -8758,7 +8755,7 @@
         <v>25</v>
       </c>
       <c r="M46" s="19" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="N46" s="19"/>
       <c r="O46" s="18"/>
@@ -8853,13 +8850,13 @@
         <v>3</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="E47" s="19" t="s">
         <v>234</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="G47" s="19" t="s">
         <v>82</v>
@@ -8868,7 +8865,7 @@
         <v>190</v>
       </c>
       <c r="I47" s="20" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="J47" s="20">
         <v>1</v>
@@ -9005,7 +9002,7 @@
         <v>513</v>
       </c>
       <c r="N48" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O48" s="35">
         <v>1</v>
@@ -9128,10 +9125,10 @@
         <v>303</v>
       </c>
       <c r="M49" s="34" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="N49" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O49" s="35">
         <v>1</v>
@@ -9257,7 +9254,7 @@
         <v>302</v>
       </c>
       <c r="N50" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O50" s="35">
         <v>1</v>
@@ -9383,7 +9380,7 @@
         <v>195</v>
       </c>
       <c r="N51" s="34" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O51" s="35">
         <v>1</v>
@@ -9479,22 +9476,22 @@
         <v>3</v>
       </c>
       <c r="D52" s="34" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E52" s="34" t="s">
         <v>234</v>
       </c>
       <c r="F52" s="34" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="G52" s="34" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="H52" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I52" s="33" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="J52" s="33">
         <v>99</v>
@@ -9503,13 +9500,13 @@
         <v>298</v>
       </c>
       <c r="L52" s="33" t="s">
+        <v>673</v>
+      </c>
+      <c r="M52" s="34" t="s">
         <v>674</v>
       </c>
-      <c r="M52" s="34" t="s">
-        <v>675</v>
-      </c>
       <c r="N52" s="34" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O52" s="35">
         <v>1</v>
@@ -9757,7 +9754,7 @@
         <v>302</v>
       </c>
       <c r="N54" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O54" s="35">
         <v>1</v>
@@ -9859,7 +9856,7 @@
         <v>235</v>
       </c>
       <c r="F55" s="34" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="G55" s="34" t="s">
         <v>490</v>
@@ -9883,7 +9880,7 @@
         <v>265</v>
       </c>
       <c r="N55" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O55" s="35">
         <v>1</v>
@@ -9979,13 +9976,13 @@
         <v>3</v>
       </c>
       <c r="D56" s="40" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E56" s="40" t="s">
         <v>235</v>
       </c>
       <c r="F56" s="40" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="G56" s="40" t="s">
         <v>103</v>
@@ -9994,7 +9991,7 @@
         <v>190</v>
       </c>
       <c r="I56" s="39" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="J56" s="39">
         <v>99</v>
@@ -10003,16 +10000,16 @@
         <v>292</v>
       </c>
       <c r="L56" s="39" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="M56" s="40" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="N56" s="40"/>
       <c r="O56" s="41"/>
       <c r="P56" s="39"/>
       <c r="Q56" s="40" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="R56" s="13"/>
       <c r="S56" s="2">
@@ -10103,13 +10100,13 @@
         <v>3</v>
       </c>
       <c r="D57" s="34" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="E57" s="34" t="s">
         <v>234</v>
       </c>
       <c r="F57" s="34" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="G57" s="34" t="s">
         <v>109</v>
@@ -10118,7 +10115,7 @@
         <v>190</v>
       </c>
       <c r="I57" s="33" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="J57" s="33"/>
       <c r="K57" s="33" t="s">
@@ -10131,7 +10128,7 @@
         <v>195</v>
       </c>
       <c r="N57" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O57" s="35">
         <v>1</v>
@@ -10351,13 +10348,13 @@
         <v>3</v>
       </c>
       <c r="D59" s="34" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="E59" s="34" t="s">
         <v>235</v>
       </c>
       <c r="F59" s="34" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="G59" s="34" t="s">
         <v>88</v>
@@ -10366,7 +10363,7 @@
         <v>190</v>
       </c>
       <c r="I59" s="33" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="J59" s="33">
         <v>2</v>
@@ -10377,7 +10374,7 @@
       <c r="L59" s="33"/>
       <c r="M59" s="34"/>
       <c r="N59" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O59" s="35">
         <v>1</v>
@@ -10505,7 +10502,7 @@
         <v>247</v>
       </c>
       <c r="N60" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O60" s="35">
         <v>1</v>
@@ -10630,7 +10627,7 @@
         <v>305</v>
       </c>
       <c r="M61" s="19" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="N61" s="19"/>
       <c r="O61" s="18"/>
@@ -10725,13 +10722,13 @@
         <v>5</v>
       </c>
       <c r="D62" s="34" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="E62" s="34" t="s">
         <v>237</v>
       </c>
       <c r="F62" s="34" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="G62" s="34" t="s">
         <v>72</v>
@@ -10740,7 +10737,7 @@
         <v>190</v>
       </c>
       <c r="I62" s="33" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="J62" s="33">
         <v>4</v>
@@ -10751,7 +10748,7 @@
       <c r="L62" s="33"/>
       <c r="M62" s="34"/>
       <c r="N62" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O62" s="35">
         <v>1</v>
@@ -10971,22 +10968,22 @@
         <v>5</v>
       </c>
       <c r="D64" s="19" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E64" s="19" t="s">
         <v>237</v>
       </c>
       <c r="F64" s="19" t="s">
+        <v>731</v>
+      </c>
+      <c r="G64" s="19" t="s">
         <v>732</v>
-      </c>
-      <c r="G64" s="19" t="s">
-        <v>733</v>
       </c>
       <c r="H64" s="19" t="s">
         <v>190</v>
       </c>
       <c r="I64" s="20" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="J64" s="20">
         <v>99</v>
@@ -10998,7 +10995,7 @@
         <v>30</v>
       </c>
       <c r="M64" s="19" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="N64" s="19"/>
       <c r="O64" s="18"/>
@@ -11093,13 +11090,13 @@
         <v>5</v>
       </c>
       <c r="D65" s="19" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="E65" s="19" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="F65" s="19" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="G65" s="19" t="s">
         <v>145</v>
@@ -11108,7 +11105,7 @@
         <v>190</v>
       </c>
       <c r="I65" s="20" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="J65" s="20">
         <v>99</v>
@@ -11120,7 +11117,7 @@
         <v>40</v>
       </c>
       <c r="M65" s="19" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="N65" s="19"/>
       <c r="O65" s="18"/>
@@ -11215,13 +11212,13 @@
         <v>5</v>
       </c>
       <c r="D66" s="19" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="E66" s="19" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="F66" s="19" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="G66" s="19" t="s">
         <v>103</v>
@@ -11230,7 +11227,7 @@
         <v>190</v>
       </c>
       <c r="I66" s="20" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="J66" s="20">
         <v>99</v>
@@ -11242,7 +11239,7 @@
         <v>40</v>
       </c>
       <c r="M66" s="19" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="N66" s="19"/>
       <c r="O66" s="18"/>
@@ -11337,13 +11334,13 @@
         <v>5</v>
       </c>
       <c r="D67" s="34" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="E67" s="34" t="s">
         <v>237</v>
       </c>
       <c r="F67" s="34" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="G67" s="34" t="s">
         <v>82</v>
@@ -11352,7 +11349,7 @@
         <v>190</v>
       </c>
       <c r="I67" s="33" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="J67" s="33">
         <v>1</v>
@@ -11364,10 +11361,10 @@
         <v>507</v>
       </c>
       <c r="M67" s="34" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="N67" s="34" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="O67" s="35">
         <v>1</v>
@@ -11490,10 +11487,10 @@
         <v>31</v>
       </c>
       <c r="M68" s="34" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="N68" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O68" s="35">
         <v>1</v>
@@ -11579,51 +11576,53 @@
       <c r="AT68" s="13"/>
     </row>
     <row r="69" spans="1:46" s="14" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="36">
-        <v>0</v>
-      </c>
-      <c r="B69" s="36">
-        <v>1</v>
-      </c>
-      <c r="C69" s="36">
+      <c r="A69" s="33">
+        <v>0</v>
+      </c>
+      <c r="B69" s="33">
+        <v>1</v>
+      </c>
+      <c r="C69" s="33">
         <v>5</v>
       </c>
-      <c r="D69" s="37" t="s">
+      <c r="D69" s="34" t="s">
         <v>334</v>
       </c>
-      <c r="E69" s="37" t="s">
+      <c r="E69" s="34" t="s">
         <v>237</v>
       </c>
-      <c r="F69" s="37" t="s">
+      <c r="F69" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="G69" s="37" t="s">
+      <c r="G69" s="34" t="s">
         <v>111</v>
       </c>
-      <c r="H69" s="37" t="s">
+      <c r="H69" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="I69" s="36" t="s">
+      <c r="I69" s="33" t="s">
         <v>561</v>
       </c>
-      <c r="J69" s="36">
+      <c r="J69" s="33">
         <v>5</v>
       </c>
-      <c r="K69" s="36" t="s">
+      <c r="K69" s="33" t="s">
         <v>298</v>
       </c>
-      <c r="L69" s="36" t="s">
-        <v>564</v>
-      </c>
-      <c r="M69" s="37" t="s">
+      <c r="L69" s="33">
+        <v>36</v>
+      </c>
+      <c r="M69" s="34" t="s">
         <v>195</v>
       </c>
-      <c r="N69" s="37" t="s">
-        <v>850</v>
-      </c>
-      <c r="O69" s="38"/>
-      <c r="P69" s="36"/>
-      <c r="Q69" s="37"/>
+      <c r="N69" s="34" t="s">
+        <v>857</v>
+      </c>
+      <c r="O69" s="35">
+        <v>1</v>
+      </c>
+      <c r="P69" s="33"/>
+      <c r="Q69" s="34"/>
       <c r="R69" s="13"/>
       <c r="S69" s="2">
         <f t="shared" si="23"/>
@@ -11672,7 +11671,7 @@
       </c>
       <c r="AE69" s="2">
         <f t="shared" si="34"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF69" s="2">
         <f t="shared" si="19"/>
@@ -11680,7 +11679,7 @@
       </c>
       <c r="AG69" s="2">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH69" s="2">
         <f t="shared" si="21"/>
@@ -11713,13 +11712,13 @@
         <v>5</v>
       </c>
       <c r="D70" s="19" t="s">
+        <v>903</v>
+      </c>
+      <c r="E70" s="19" t="s">
+        <v>840</v>
+      </c>
+      <c r="F70" s="19" t="s">
         <v>904</v>
-      </c>
-      <c r="E70" s="19" t="s">
-        <v>841</v>
-      </c>
-      <c r="F70" s="19" t="s">
-        <v>905</v>
       </c>
       <c r="G70" s="19" t="s">
         <v>72</v>
@@ -11728,7 +11727,7 @@
         <v>190</v>
       </c>
       <c r="I70" s="20" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="J70" s="20">
         <v>4</v>
@@ -11740,7 +11739,7 @@
         <v>45</v>
       </c>
       <c r="M70" s="19" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="N70" s="19"/>
       <c r="O70" s="18"/>
@@ -11835,13 +11834,13 @@
         <v>5</v>
       </c>
       <c r="D71" s="34" t="s">
+        <v>815</v>
+      </c>
+      <c r="E71" s="34" t="s">
         <v>816</v>
       </c>
-      <c r="E71" s="34" t="s">
-        <v>817</v>
-      </c>
       <c r="F71" s="34" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="G71" s="34" t="s">
         <v>72</v>
@@ -11850,7 +11849,7 @@
         <v>190</v>
       </c>
       <c r="I71" s="33" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="J71" s="33"/>
       <c r="K71" s="33" t="s">
@@ -11860,10 +11859,10 @@
         <v>45</v>
       </c>
       <c r="M71" s="34" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="N71" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O71" s="35">
         <v>1</v>
@@ -11983,13 +11982,13 @@
         <v>291</v>
       </c>
       <c r="L72" s="36" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="M72" s="37" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="N72" s="37" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O72" s="38"/>
       <c r="P72" s="36"/>
@@ -12083,22 +12082,22 @@
         <v>5</v>
       </c>
       <c r="D73" s="34" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="E73" s="34" t="s">
         <v>237</v>
       </c>
       <c r="F73" s="34" t="s">
+        <v>808</v>
+      </c>
+      <c r="G73" s="34" t="s">
         <v>809</v>
-      </c>
-      <c r="G73" s="34" t="s">
-        <v>810</v>
       </c>
       <c r="H73" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I73" s="33" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="J73" s="33">
         <v>1</v>
@@ -12113,7 +12112,7 @@
         <v>513</v>
       </c>
       <c r="N73" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O73" s="35">
         <v>1</v>
@@ -12209,10 +12208,10 @@
         <v>5</v>
       </c>
       <c r="D74" s="34" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="E74" s="34" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="F74" s="34" t="s">
         <v>68</v>
@@ -12224,7 +12223,7 @@
         <v>190</v>
       </c>
       <c r="I74" s="33" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="J74" s="33">
         <v>2</v>
@@ -12239,7 +12238,7 @@
         <v>513</v>
       </c>
       <c r="N74" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O74" s="35">
         <v>1</v>
@@ -12606,10 +12605,10 @@
         <v>70</v>
       </c>
       <c r="M77" s="34" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="N77" s="34" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="O77" s="35">
         <v>1</v>
@@ -12827,13 +12826,13 @@
         <v>6</v>
       </c>
       <c r="D79" s="19" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="E79" s="19" t="s">
         <v>241</v>
       </c>
       <c r="F79" s="19" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="G79" s="19" t="s">
         <v>88</v>
@@ -12842,7 +12841,7 @@
         <v>190</v>
       </c>
       <c r="I79" s="20" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="J79" s="20">
         <v>2</v>
@@ -12854,7 +12853,7 @@
         <v>301</v>
       </c>
       <c r="M79" s="19" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="N79" s="19"/>
       <c r="O79" s="18"/>
@@ -12949,13 +12948,13 @@
         <v>6</v>
       </c>
       <c r="D80" s="19" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="E80" s="19" t="s">
         <v>241</v>
       </c>
       <c r="F80" s="19" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="G80" s="19" t="s">
         <v>82</v>
@@ -12964,7 +12963,7 @@
         <v>190</v>
       </c>
       <c r="I80" s="20" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="J80" s="20">
         <v>1</v>
@@ -12976,13 +12975,13 @@
         <v>301</v>
       </c>
       <c r="M80" s="19" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="N80" s="19"/>
       <c r="O80" s="18"/>
       <c r="P80" s="20"/>
       <c r="Q80" s="19" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="R80" s="13"/>
       <c r="S80" s="2">
@@ -13103,7 +13102,7 @@
         <v>508</v>
       </c>
       <c r="N81" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O81" s="35">
         <v>1</v>
@@ -13199,22 +13198,22 @@
         <v>6</v>
       </c>
       <c r="D82" s="34" t="s">
+        <v>569</v>
+      </c>
+      <c r="E82" s="34" t="s">
         <v>570</v>
       </c>
-      <c r="E82" s="34" t="s">
+      <c r="F82" s="34" t="s">
         <v>571</v>
       </c>
-      <c r="F82" s="34" t="s">
-        <v>572</v>
-      </c>
       <c r="G82" s="34" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="H82" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I82" s="33" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="J82" s="33">
         <v>1</v>
@@ -13229,7 +13228,7 @@
         <v>103</v>
       </c>
       <c r="N82" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O82" s="35">
         <v>1</v>
@@ -13357,7 +13356,7 @@
         <v>248</v>
       </c>
       <c r="N83" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O83" s="35">
         <v>1</v>
@@ -13453,13 +13452,13 @@
         <v>6</v>
       </c>
       <c r="D84" s="34" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="E84" s="34" t="s">
         <v>519</v>
       </c>
       <c r="F84" s="34" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="G84" s="34" t="s">
         <v>495</v>
@@ -13468,7 +13467,7 @@
         <v>190</v>
       </c>
       <c r="I84" s="33" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="J84" s="33">
         <v>2</v>
@@ -13483,7 +13482,7 @@
         <v>103</v>
       </c>
       <c r="N84" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O84" s="35">
         <v>1</v>
@@ -13581,13 +13580,13 @@
         <v>6</v>
       </c>
       <c r="D85" s="34" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="E85" s="34" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="F85" s="34" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="G85" s="34" t="s">
         <v>144</v>
@@ -13596,7 +13595,7 @@
         <v>190</v>
       </c>
       <c r="I85" s="33" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="J85" s="33">
         <v>99</v>
@@ -13608,10 +13607,10 @@
         <v>507</v>
       </c>
       <c r="M85" s="34" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="N85" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O85" s="35">
         <v>1</v>
@@ -13707,13 +13706,13 @@
         <v>6</v>
       </c>
       <c r="D86" s="34" t="s">
+        <v>880</v>
+      </c>
+      <c r="E86" s="34" t="s">
         <v>881</v>
       </c>
-      <c r="E86" s="34" t="s">
+      <c r="F86" s="34" t="s">
         <v>882</v>
-      </c>
-      <c r="F86" s="34" t="s">
-        <v>883</v>
       </c>
       <c r="G86" s="34" t="s">
         <v>88</v>
@@ -13722,7 +13721,7 @@
         <v>190</v>
       </c>
       <c r="I86" s="33" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="J86" s="33">
         <v>2</v>
@@ -13734,10 +13733,10 @@
         <v>45</v>
       </c>
       <c r="M86" s="34" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="N86" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O86" s="35">
         <v>1</v>
@@ -13830,22 +13829,22 @@
         <v>6</v>
       </c>
       <c r="D87" s="34" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="E87" s="34" t="s">
         <v>481</v>
       </c>
       <c r="F87" s="34" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="G87" s="34" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="H87" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I87" s="33" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="J87" s="33">
         <v>1</v>
@@ -13860,7 +13859,7 @@
         <v>516</v>
       </c>
       <c r="N87" s="34" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O87" s="35">
         <v>1</v>
@@ -13953,7 +13952,7 @@
         <v>6</v>
       </c>
       <c r="D88" s="34" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="E88" s="34" t="s">
         <v>481</v>
@@ -13983,7 +13982,7 @@
         <v>516</v>
       </c>
       <c r="N88" s="34" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O88" s="35">
         <v>1</v>
@@ -14109,7 +14108,7 @@
         <v>248</v>
       </c>
       <c r="N89" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O89" s="35">
         <v>1</v>
@@ -14205,20 +14204,20 @@
         <v>6</v>
       </c>
       <c r="D90" s="34" t="s">
+        <v>862</v>
+      </c>
+      <c r="E90" s="34" t="s">
         <v>863</v>
       </c>
-      <c r="E90" s="34" t="s">
+      <c r="F90" s="34" t="s">
         <v>864</v>
-      </c>
-      <c r="F90" s="34" t="s">
-        <v>865</v>
       </c>
       <c r="G90" s="34"/>
       <c r="H90" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I90" s="33" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="J90" s="33"/>
       <c r="K90" s="33" t="s">
@@ -14227,7 +14226,7 @@
       <c r="L90" s="33"/>
       <c r="M90" s="34"/>
       <c r="N90" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O90" s="35">
         <v>1</v>
@@ -14340,7 +14339,7 @@
         <v>190</v>
       </c>
       <c r="I91" s="33" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="J91" s="33">
         <v>5</v>
@@ -14355,7 +14354,7 @@
         <v>195</v>
       </c>
       <c r="N91" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O91" s="35">
         <v>1</v>
@@ -14451,7 +14450,7 @@
         <v>6</v>
       </c>
       <c r="D92" s="34" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="E92" s="34" t="s">
         <v>519</v>
@@ -14478,10 +14477,10 @@
         <v>305</v>
       </c>
       <c r="M92" s="34" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="N92" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O92" s="35">
         <v>1</v>
@@ -14705,7 +14704,7 @@
         <v>40</v>
       </c>
       <c r="F94" s="40" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="G94" s="40" t="s">
         <v>103</v>
@@ -14726,10 +14725,10 @@
         <v>305</v>
       </c>
       <c r="M94" s="40" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="N94" s="40" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O94" s="41">
         <v>1</v>
@@ -14855,7 +14854,7 @@
         <v>309</v>
       </c>
       <c r="N95" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O95" s="35">
         <v>1</v>
@@ -14983,7 +14982,7 @@
         <v>309</v>
       </c>
       <c r="N96" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O96" s="35">
         <v>1</v>
@@ -15111,7 +15110,7 @@
         <v>309</v>
       </c>
       <c r="N97" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O97" s="35">
         <v>1</v>
@@ -15120,7 +15119,7 @@
         <v>1</v>
       </c>
       <c r="Q97" s="34" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="R97" s="13"/>
       <c r="S97" s="2">
@@ -15217,7 +15216,7 @@
         <v>40</v>
       </c>
       <c r="F98" s="34" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="G98" s="34" t="s">
         <v>137</v>
@@ -15226,7 +15225,7 @@
         <v>190</v>
       </c>
       <c r="I98" s="33" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="J98" s="33">
         <v>99</v>
@@ -15241,7 +15240,7 @@
         <v>268</v>
       </c>
       <c r="N98" s="34" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O98" s="35">
         <v>1</v>
@@ -15367,7 +15366,7 @@
         <v>268</v>
       </c>
       <c r="N99" s="34" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O99" s="35">
         <v>1</v>
@@ -15463,13 +15462,13 @@
         <v>7</v>
       </c>
       <c r="D100" s="34" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="E100" s="34" t="s">
         <v>40</v>
       </c>
       <c r="F100" s="34" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="G100" s="34" t="s">
         <v>72</v>
@@ -15478,7 +15477,7 @@
         <v>190</v>
       </c>
       <c r="I100" s="33" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="J100" s="33">
         <v>3</v>
@@ -15490,10 +15489,10 @@
         <v>28</v>
       </c>
       <c r="M100" s="34" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="N100" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O100" s="35">
         <v>1</v>
@@ -15592,7 +15591,7 @@
         <v>335</v>
       </c>
       <c r="E101" s="34" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F101" s="34" t="s">
         <v>356</v>
@@ -15619,7 +15618,7 @@
         <v>195</v>
       </c>
       <c r="N101" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O101" s="35">
         <v>1</v>
@@ -15715,22 +15714,22 @@
         <v>7</v>
       </c>
       <c r="D102" s="19" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E102" s="19" t="s">
         <v>40</v>
       </c>
       <c r="F102" s="19" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="G102" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="H102" s="19" t="s">
         <v>190</v>
       </c>
       <c r="I102" s="20" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="J102" s="20">
         <v>99</v>
@@ -15742,7 +15741,7 @@
         <v>306</v>
       </c>
       <c r="M102" s="19" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="N102" s="19"/>
       <c r="O102" s="18"/>
@@ -15837,13 +15836,13 @@
         <v>7</v>
       </c>
       <c r="D103" s="34" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="E103" s="34" t="s">
         <v>40</v>
       </c>
       <c r="F103" s="34" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="G103" s="34" t="s">
         <v>72</v>
@@ -15852,7 +15851,7 @@
         <v>190</v>
       </c>
       <c r="I103" s="33" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="J103" s="33">
         <v>3</v>
@@ -15864,10 +15863,10 @@
         <v>30</v>
       </c>
       <c r="M103" s="34" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="N103" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O103" s="35">
         <v>1</v>
@@ -15993,7 +15992,7 @@
         <v>563</v>
       </c>
       <c r="N104" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O104" s="35">
         <v>1</v>
@@ -16079,51 +16078,53 @@
       <c r="AT104" s="13"/>
     </row>
     <row r="105" spans="1:46" s="14" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="36">
-        <v>0</v>
-      </c>
-      <c r="B105" s="36">
-        <v>1</v>
-      </c>
-      <c r="C105" s="36">
+      <c r="A105" s="33">
+        <v>0</v>
+      </c>
+      <c r="B105" s="33">
+        <v>1</v>
+      </c>
+      <c r="C105" s="33">
         <v>7</v>
       </c>
-      <c r="D105" s="37" t="s">
+      <c r="D105" s="34" t="s">
         <v>220</v>
       </c>
-      <c r="E105" s="37" t="s">
+      <c r="E105" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="F105" s="37" t="s">
+      <c r="F105" s="34" t="s">
         <v>178</v>
       </c>
-      <c r="G105" s="37" t="s">
+      <c r="G105" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="H105" s="37" t="s">
+      <c r="H105" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="I105" s="36" t="s">
+      <c r="I105" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="J105" s="36">
-        <v>1</v>
-      </c>
-      <c r="K105" s="36" t="s">
+      <c r="J105" s="33">
+        <v>1</v>
+      </c>
+      <c r="K105" s="33" t="s">
         <v>294</v>
       </c>
-      <c r="L105" s="36" t="s">
+      <c r="L105" s="33" t="s">
         <v>305</v>
       </c>
-      <c r="M105" s="37" t="s">
+      <c r="M105" s="34" t="s">
         <v>249</v>
       </c>
-      <c r="N105" s="37" t="s">
+      <c r="N105" s="34" t="s">
         <v>879</v>
       </c>
-      <c r="O105" s="38"/>
-      <c r="P105" s="36"/>
-      <c r="Q105" s="37"/>
+      <c r="O105" s="35">
+        <v>1</v>
+      </c>
+      <c r="P105" s="33"/>
+      <c r="Q105" s="34"/>
       <c r="R105" s="13"/>
       <c r="S105" s="2">
         <f t="shared" si="39"/>
@@ -16172,7 +16173,7 @@
       </c>
       <c r="AE105" s="2">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF105" s="2">
         <f t="shared" si="35"/>
@@ -16180,7 +16181,7 @@
       </c>
       <c r="AG105" s="2">
         <f t="shared" si="36"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH105" s="2">
         <f t="shared" si="37"/>
@@ -16213,13 +16214,13 @@
         <v>1</v>
       </c>
       <c r="D106" s="34" t="s">
+        <v>686</v>
+      </c>
+      <c r="E106" s="34" t="s">
         <v>687</v>
       </c>
-      <c r="E106" s="34" t="s">
+      <c r="F106" s="34" t="s">
         <v>688</v>
-      </c>
-      <c r="F106" s="34" t="s">
-        <v>689</v>
       </c>
       <c r="G106" s="34" t="s">
         <v>88</v>
@@ -16228,7 +16229,7 @@
         <v>190</v>
       </c>
       <c r="I106" s="33" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="J106" s="33">
         <v>2</v>
@@ -16240,10 +16241,10 @@
         <v>7</v>
       </c>
       <c r="M106" s="34" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="N106" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O106" s="35">
         <v>1</v>
@@ -16341,13 +16342,13 @@
         <v>1</v>
       </c>
       <c r="D107" s="34" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="E107" s="34" t="s">
         <v>69</v>
       </c>
       <c r="F107" s="34" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="G107" s="34" t="s">
         <v>88</v>
@@ -16356,7 +16357,7 @@
         <v>190</v>
       </c>
       <c r="I107" s="33" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="J107" s="33">
         <v>2</v>
@@ -16368,10 +16369,10 @@
         <v>5</v>
       </c>
       <c r="M107" s="34" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="N107" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O107" s="35">
         <v>1</v>
@@ -16380,7 +16381,7 @@
         <v>1</v>
       </c>
       <c r="Q107" s="34" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="R107" s="13"/>
       <c r="S107" s="2">
@@ -16471,13 +16472,13 @@
         <v>1</v>
       </c>
       <c r="D108" s="34" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E108" s="34" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F108" s="34" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="G108" s="34" t="s">
         <v>82</v>
@@ -16501,7 +16502,7 @@
         <v>193</v>
       </c>
       <c r="N108" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O108" s="35">
         <v>1</v>
@@ -16510,7 +16511,7 @@
         <v>1</v>
       </c>
       <c r="Q108" s="34" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="R108" s="13"/>
       <c r="S108" s="2">
@@ -16601,13 +16602,13 @@
         <v>1</v>
       </c>
       <c r="D109" s="34" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="E109" s="34" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="F109" s="34" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="G109" s="34" t="s">
         <v>144</v>
@@ -16616,7 +16617,7 @@
         <v>190</v>
       </c>
       <c r="I109" s="33" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="J109" s="33">
         <v>99</v>
@@ -16631,7 +16632,7 @@
         <v>193</v>
       </c>
       <c r="N109" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O109" s="35">
         <v>1</v>
@@ -16729,13 +16730,13 @@
         <v>1</v>
       </c>
       <c r="D110" s="34" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="E110" s="34" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="F110" s="34" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="G110" s="34" t="s">
         <v>103</v>
@@ -16744,7 +16745,7 @@
         <v>190</v>
       </c>
       <c r="I110" s="33" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="J110" s="33">
         <v>99</v>
@@ -16756,10 +16757,10 @@
         <v>9</v>
       </c>
       <c r="M110" s="34" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="N110" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O110" s="35">
         <v>1</v>
@@ -17226,7 +17227,7 @@
         <v>166</v>
       </c>
       <c r="E114" s="34" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F114" s="34" t="s">
         <v>165</v>
@@ -17253,7 +17254,7 @@
         <v>193</v>
       </c>
       <c r="N114" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O114" s="35">
         <v>1</v>
@@ -17379,7 +17380,7 @@
         <v>193</v>
       </c>
       <c r="N115" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O115" s="35">
         <v>1</v>
@@ -17483,16 +17484,16 @@
         <v>61</v>
       </c>
       <c r="F116" s="34" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="G116" s="34" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="H116" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I116" s="33" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="J116" s="33">
         <v>99</v>
@@ -17507,7 +17508,7 @@
         <v>193</v>
       </c>
       <c r="N116" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O116" s="35">
         <v>1</v>
@@ -17757,7 +17758,7 @@
         <v>193</v>
       </c>
       <c r="N118" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O118" s="35">
         <v>1</v>
@@ -17855,13 +17856,13 @@
         <v>1</v>
       </c>
       <c r="D119" s="34" t="s">
+        <v>566</v>
+      </c>
+      <c r="E119" s="34" t="s">
+        <v>687</v>
+      </c>
+      <c r="F119" s="34" t="s">
         <v>567</v>
-      </c>
-      <c r="E119" s="34" t="s">
-        <v>688</v>
-      </c>
-      <c r="F119" s="34" t="s">
-        <v>568</v>
       </c>
       <c r="G119" s="34" t="s">
         <v>88</v>
@@ -17870,7 +17871,7 @@
         <v>190</v>
       </c>
       <c r="I119" s="33" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="J119" s="33">
         <v>2</v>
@@ -17882,10 +17883,10 @@
         <v>9</v>
       </c>
       <c r="M119" s="34" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="N119" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O119" s="35">
         <v>1</v>
@@ -18132,10 +18133,10 @@
         <v>303</v>
       </c>
       <c r="M121" s="34" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="N121" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O121" s="35">
         <v>1</v>
@@ -18231,22 +18232,22 @@
         <v>2</v>
       </c>
       <c r="D122" s="34" t="s">
+        <v>820</v>
+      </c>
+      <c r="E122" s="34" t="s">
+        <v>753</v>
+      </c>
+      <c r="F122" s="34" t="s">
         <v>821</v>
       </c>
-      <c r="E122" s="34" t="s">
-        <v>754</v>
-      </c>
-      <c r="F122" s="34" t="s">
+      <c r="G122" s="34" t="s">
         <v>822</v>
-      </c>
-      <c r="G122" s="34" t="s">
-        <v>823</v>
       </c>
       <c r="H122" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I122" s="33" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="J122" s="33"/>
       <c r="K122" s="33" t="s">
@@ -18256,10 +18257,10 @@
         <v>30</v>
       </c>
       <c r="M122" s="34" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="N122" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O122" s="35">
         <v>1</v>
@@ -18382,10 +18383,10 @@
         <v>310</v>
       </c>
       <c r="M123" s="34" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="N123" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O123" s="35">
         <v>1</v>
@@ -18483,13 +18484,13 @@
         <v>2</v>
       </c>
       <c r="D124" s="34" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="E124" s="34" t="s">
         <v>241</v>
       </c>
       <c r="F124" s="34" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="G124" s="34" t="s">
         <v>160</v>
@@ -18498,7 +18499,7 @@
         <v>190</v>
       </c>
       <c r="I124" s="33" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="J124" s="33">
         <v>1</v>
@@ -18507,13 +18508,13 @@
         <v>293</v>
       </c>
       <c r="L124" s="33" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="M124" s="34" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="N124" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O124" s="35">
         <v>1</v>
@@ -18859,16 +18860,16 @@
         <v>382</v>
       </c>
       <c r="F127" s="19" t="s">
+        <v>643</v>
+      </c>
+      <c r="G127" s="19" t="s">
         <v>644</v>
-      </c>
-      <c r="G127" s="19" t="s">
-        <v>645</v>
       </c>
       <c r="H127" s="19" t="s">
         <v>190</v>
       </c>
       <c r="I127" s="20" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="J127" s="20">
         <v>99</v>
@@ -18880,7 +18881,7 @@
         <v>306</v>
       </c>
       <c r="M127" s="19" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="N127" s="19"/>
       <c r="O127" s="18"/>
@@ -18981,7 +18982,7 @@
         <v>382</v>
       </c>
       <c r="F128" s="19" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G128" s="19" t="s">
         <v>204</v>
@@ -19002,7 +19003,7 @@
         <v>306</v>
       </c>
       <c r="M128" s="19" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="N128" s="19"/>
       <c r="O128" s="18"/>
@@ -19463,18 +19464,18 @@
         <v>2</v>
       </c>
       <c r="D132" s="34" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="E132" s="34"/>
       <c r="F132" s="34" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G132" s="34"/>
       <c r="H132" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I132" s="33" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="J132" s="33"/>
       <c r="K132" s="33" t="s">
@@ -19484,10 +19485,10 @@
         <v>22</v>
       </c>
       <c r="M132" s="34" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="N132" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O132" s="35">
         <v>1</v>
@@ -19612,10 +19613,10 @@
         <v>307</v>
       </c>
       <c r="M133" s="34" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="N133" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O133" s="35">
         <v>1</v>
@@ -19728,7 +19729,7 @@
         <v>190</v>
       </c>
       <c r="I134" s="33" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="J134" s="33">
         <v>5</v>
@@ -19743,7 +19744,7 @@
         <v>456</v>
       </c>
       <c r="N134" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O134" s="35">
         <v>1</v>
@@ -19961,13 +19962,13 @@
         <v>2</v>
       </c>
       <c r="D136" s="37" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E136" s="37" t="s">
         <v>279</v>
       </c>
       <c r="F136" s="37" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="G136" s="37" t="s">
         <v>145</v>
@@ -19976,7 +19977,7 @@
         <v>190</v>
       </c>
       <c r="I136" s="36" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="J136" s="36">
         <v>99</v>
@@ -19988,10 +19989,10 @@
         <v>505</v>
       </c>
       <c r="M136" s="37" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="N136" s="37" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O136" s="38"/>
       <c r="P136" s="36"/>
@@ -20109,13 +20110,13 @@
         <v>293</v>
       </c>
       <c r="L137" s="33" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="M137" s="34" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="N137" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O137" s="35">
         <v>1</v>
@@ -20243,7 +20244,7 @@
         <v>103</v>
       </c>
       <c r="N138" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O138" s="35">
         <v>1</v>
@@ -20341,13 +20342,13 @@
         <v>3</v>
       </c>
       <c r="D139" s="34" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="E139" s="34" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="F139" s="34" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="G139" s="34" t="s">
         <v>496</v>
@@ -20356,7 +20357,7 @@
         <v>190</v>
       </c>
       <c r="I139" s="33" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="J139" s="33">
         <v>1</v>
@@ -20371,7 +20372,7 @@
         <v>103</v>
       </c>
       <c r="N139" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O139" s="35">
         <v>1</v>
@@ -20499,7 +20500,7 @@
         <v>103</v>
       </c>
       <c r="N140" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O140" s="35">
         <v>1</v>
@@ -20597,13 +20598,13 @@
         <v>3</v>
       </c>
       <c r="D141" s="34" t="s">
+        <v>873</v>
+      </c>
+      <c r="E141" s="34" t="s">
+        <v>872</v>
+      </c>
+      <c r="F141" s="34" t="s">
         <v>874</v>
-      </c>
-      <c r="E141" s="34" t="s">
-        <v>873</v>
-      </c>
-      <c r="F141" s="34" t="s">
-        <v>875</v>
       </c>
       <c r="G141" s="34" t="s">
         <v>137</v>
@@ -20612,7 +20613,7 @@
         <v>190</v>
       </c>
       <c r="I141" s="33" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="J141" s="33">
         <v>1</v>
@@ -20623,7 +20624,7 @@
       <c r="L141" s="33"/>
       <c r="M141" s="34"/>
       <c r="N141" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O141" s="35">
         <v>1</v>
@@ -20721,13 +20722,13 @@
         <v>3</v>
       </c>
       <c r="D142" s="34" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="E142" s="34" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="F142" s="34" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="G142" s="34" t="s">
         <v>83</v>
@@ -20736,7 +20737,7 @@
         <v>190</v>
       </c>
       <c r="I142" s="33" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J142" s="33">
         <v>1</v>
@@ -20751,7 +20752,7 @@
         <v>103</v>
       </c>
       <c r="N142" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O142" s="35">
         <v>1</v>
@@ -20760,7 +20761,7 @@
         <v>1</v>
       </c>
       <c r="Q142" s="34" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="R142" s="13"/>
       <c r="S142" s="2">
@@ -20881,7 +20882,7 @@
         <v>314</v>
       </c>
       <c r="N143" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O143" s="35">
         <v>1</v>
@@ -21231,7 +21232,7 @@
         <v>37</v>
       </c>
       <c r="F146" s="37" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="G146" s="37" t="s">
         <v>72</v>
@@ -21252,10 +21253,10 @@
         <v>305</v>
       </c>
       <c r="M146" s="37" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="N146" s="37" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O146" s="38"/>
       <c r="P146" s="36"/>
@@ -21349,13 +21350,13 @@
         <v>4</v>
       </c>
       <c r="D147" s="19" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="E147" s="19" t="s">
         <v>411</v>
       </c>
       <c r="F147" s="19" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G147" s="19" t="s">
         <v>495</v>
@@ -21376,7 +21377,7 @@
         <v>307</v>
       </c>
       <c r="M147" s="19" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="N147" s="19"/>
       <c r="O147" s="18"/>
@@ -21471,13 +21472,13 @@
         <v>4</v>
       </c>
       <c r="D148" s="34" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="E148" s="34" t="s">
         <v>411</v>
       </c>
       <c r="F148" s="34" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="G148" s="34" t="s">
         <v>110</v>
@@ -21486,7 +21487,7 @@
         <v>190</v>
       </c>
       <c r="I148" s="33" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="J148" s="33">
         <v>3</v>
@@ -21498,10 +21499,10 @@
         <v>305</v>
       </c>
       <c r="M148" s="34" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="N148" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O148" s="35">
         <v>1</v>
@@ -21627,7 +21628,7 @@
         <v>514</v>
       </c>
       <c r="N149" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O149" s="35">
         <v>1</v>
@@ -21729,7 +21730,7 @@
         <v>30</v>
       </c>
       <c r="F150" s="34" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G150" s="34" t="s">
         <v>101</v>
@@ -21750,10 +21751,10 @@
         <v>310</v>
       </c>
       <c r="M150" s="34" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="N150" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O150" s="35">
         <v>1</v>
@@ -21878,10 +21879,10 @@
         <v>310</v>
       </c>
       <c r="M151" s="34" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="N151" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O151" s="35">
         <v>1</v>
@@ -22125,10 +22126,10 @@
         <v>307</v>
       </c>
       <c r="M153" s="40" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="N153" s="40" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="O153" s="41"/>
       <c r="P153" s="39"/>
@@ -22222,20 +22223,20 @@
         <v>4</v>
       </c>
       <c r="D154" s="19" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="E154" s="19" t="s">
         <v>410</v>
       </c>
       <c r="F154" s="19" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="G154" s="19"/>
       <c r="H154" s="19" t="s">
         <v>190</v>
       </c>
       <c r="I154" s="20" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="J154" s="20"/>
       <c r="K154" s="20" t="s">
@@ -22245,7 +22246,7 @@
         <v>20</v>
       </c>
       <c r="M154" s="19" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="N154" s="19"/>
       <c r="O154" s="18"/>
@@ -22367,7 +22368,7 @@
         <v>30</v>
       </c>
       <c r="M155" s="19" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="N155" s="19"/>
       <c r="O155" s="18"/>
@@ -22462,13 +22463,13 @@
         <v>5</v>
       </c>
       <c r="D156" s="34" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E156" s="34" t="s">
         <v>532</v>
       </c>
       <c r="F156" s="34" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="G156" s="34" t="s">
         <v>82</v>
@@ -22477,7 +22478,7 @@
         <v>190</v>
       </c>
       <c r="I156" s="33" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="J156" s="33"/>
       <c r="K156" s="33" t="s">
@@ -22487,10 +22488,10 @@
         <v>40</v>
       </c>
       <c r="M156" s="34" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="N156" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O156" s="35">
         <v>1</v>
@@ -22586,22 +22587,22 @@
         <v>5</v>
       </c>
       <c r="D157" s="34" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="E157" s="34" t="s">
         <v>477</v>
       </c>
       <c r="F157" s="34" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="G157" s="34" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="H157" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I157" s="33" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="J157" s="33">
         <v>2</v>
@@ -22613,10 +22614,10 @@
         <v>305</v>
       </c>
       <c r="M157" s="34" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="N157" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O157" s="35">
         <v>1</v>
@@ -22834,13 +22835,13 @@
         <v>5</v>
       </c>
       <c r="D159" s="34" t="s">
+        <v>839</v>
+      </c>
+      <c r="E159" s="34" t="s">
         <v>840</v>
       </c>
-      <c r="E159" s="34" t="s">
+      <c r="F159" s="34" t="s">
         <v>841</v>
-      </c>
-      <c r="F159" s="34" t="s">
-        <v>842</v>
       </c>
       <c r="G159" s="34" t="s">
         <v>129</v>
@@ -22849,7 +22850,7 @@
         <v>190</v>
       </c>
       <c r="I159" s="33" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="J159" s="33">
         <v>99</v>
@@ -22861,10 +22862,10 @@
         <v>40</v>
       </c>
       <c r="M159" s="34" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="N159" s="34" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="O159" s="35">
         <v>1</v>
@@ -22960,20 +22961,20 @@
         <v>5</v>
       </c>
       <c r="D160" s="34" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="E160" s="34" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="F160" s="34" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="G160" s="34"/>
       <c r="H160" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I160" s="33" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="J160" s="33"/>
       <c r="K160" s="33" t="s">
@@ -22983,10 +22984,10 @@
         <v>35</v>
       </c>
       <c r="M160" s="34" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="N160" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O160" s="35">
         <v>1</v>
@@ -23112,7 +23113,7 @@
         <v>461</v>
       </c>
       <c r="N161" s="34" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O161" s="35">
         <v>1</v>
@@ -23598,10 +23599,10 @@
         <v>305</v>
       </c>
       <c r="M165" s="34" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="N165" s="34" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="O165" s="35">
         <v>1</v>
@@ -23849,7 +23850,7 @@
         <v>103</v>
       </c>
       <c r="N167" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O167" s="35">
         <v>1</v>
@@ -23953,7 +23954,7 @@
         <v>87</v>
       </c>
       <c r="F168" s="19" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="G168" s="19" t="s">
         <v>100</v>
@@ -24099,7 +24100,7 @@
         <v>196</v>
       </c>
       <c r="N169" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O169" s="35">
         <v>1</v>
@@ -24203,7 +24204,7 @@
         <v>38</v>
       </c>
       <c r="F170" s="34" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="G170" s="34" t="s">
         <v>82</v>
@@ -24227,7 +24228,7 @@
         <v>196</v>
       </c>
       <c r="N170" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O170" s="35">
         <v>1</v>
@@ -24355,7 +24356,7 @@
         <v>196</v>
       </c>
       <c r="N171" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O171" s="35">
         <v>1</v>
@@ -24459,16 +24460,16 @@
         <v>38</v>
       </c>
       <c r="F172" s="34" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="G172" s="34" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="H172" s="34" t="s">
         <v>190</v>
       </c>
       <c r="I172" s="33" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="J172" s="33">
         <v>1</v>
@@ -24483,7 +24484,7 @@
         <v>196</v>
       </c>
       <c r="N172" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O172" s="35">
         <v>1</v>
@@ -24611,7 +24612,7 @@
         <v>196</v>
       </c>
       <c r="N173" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O173" s="35">
         <v>1</v>
@@ -24739,7 +24740,7 @@
         <v>196</v>
       </c>
       <c r="N174" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O174" s="35">
         <v>1</v>
@@ -24841,7 +24842,7 @@
         <v>38</v>
       </c>
       <c r="F175" s="34" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="G175" s="34" t="s">
         <v>145</v>
@@ -24850,7 +24851,7 @@
         <v>190</v>
       </c>
       <c r="I175" s="33" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="J175" s="33">
         <v>99</v>
@@ -24865,7 +24866,7 @@
         <v>196</v>
       </c>
       <c r="N175" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O175" s="35">
         <v>1</v>
@@ -25479,7 +25480,7 @@
         <v>196</v>
       </c>
       <c r="N180" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O180" s="35">
         <v>1</v>
@@ -25607,7 +25608,7 @@
         <v>196</v>
       </c>
       <c r="N181" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O181" s="35">
         <v>1</v>
@@ -25735,7 +25736,7 @@
         <v>196</v>
       </c>
       <c r="N182" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O182" s="35">
         <v>1</v>
@@ -25860,7 +25861,7 @@
         <v>196</v>
       </c>
       <c r="N183" s="37" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="O183" s="38"/>
       <c r="P183" s="36"/>
@@ -26228,7 +26229,7 @@
         <v>103</v>
       </c>
       <c r="N186" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O186" s="35">
         <v>1</v>
@@ -26478,7 +26479,7 @@
         <v>196</v>
       </c>
       <c r="N188" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O188" s="35">
         <v>1</v>
@@ -26948,7 +26949,7 @@
         <v>38</v>
       </c>
       <c r="F192" s="34" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="G192" s="34" t="s">
         <v>72</v>
@@ -26972,7 +26973,7 @@
         <v>196</v>
       </c>
       <c r="N192" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O192" s="35">
         <v>1</v>
@@ -27100,7 +27101,7 @@
         <v>196</v>
       </c>
       <c r="N193" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O193" s="35">
         <v>1</v>
@@ -27228,7 +27229,7 @@
         <v>196</v>
       </c>
       <c r="N194" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O194" s="35">
         <v>1</v>
@@ -27356,7 +27357,7 @@
         <v>384</v>
       </c>
       <c r="N195" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O195" s="35">
         <v>1</v>
@@ -27460,7 +27461,7 @@
         <v>55</v>
       </c>
       <c r="F196" s="34" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="G196" s="34" t="s">
         <v>72</v>
@@ -27469,7 +27470,7 @@
         <v>190</v>
       </c>
       <c r="I196" s="33" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="J196" s="33">
         <v>4</v>
@@ -27484,7 +27485,7 @@
         <v>384</v>
       </c>
       <c r="N196" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O196" s="35">
         <v>1</v>
@@ -27948,13 +27949,13 @@
         <v>7</v>
       </c>
       <c r="D200" s="34" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="E200" s="34" t="s">
         <v>38</v>
       </c>
       <c r="F200" s="34" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="G200" s="34" t="s">
         <v>72</v>
@@ -27963,7 +27964,7 @@
         <v>190</v>
       </c>
       <c r="I200" s="33" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="J200" s="33">
         <v>4</v>
@@ -27978,7 +27979,7 @@
         <v>103</v>
       </c>
       <c r="N200" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O200" s="35">
         <v>1</v>
@@ -28076,13 +28077,13 @@
         <v>7</v>
       </c>
       <c r="D201" s="34" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="E201" s="34" t="s">
         <v>38</v>
       </c>
       <c r="F201" s="34" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="G201" s="34" t="s">
         <v>100</v>
@@ -28091,7 +28092,7 @@
         <v>190</v>
       </c>
       <c r="I201" s="33" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="J201" s="33">
         <v>99</v>
@@ -28106,7 +28107,7 @@
         <v>103</v>
       </c>
       <c r="N201" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O201" s="35">
         <v>1</v>
@@ -28210,7 +28211,7 @@
         <v>38</v>
       </c>
       <c r="F202" s="34" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="G202" s="34" t="s">
         <v>82</v>
@@ -28234,7 +28235,7 @@
         <v>196</v>
       </c>
       <c r="N202" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O202" s="35">
         <v>1</v>
@@ -28360,7 +28361,7 @@
         <v>196</v>
       </c>
       <c r="N203" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O203" s="35">
         <v>1</v>
@@ -28486,7 +28487,7 @@
         <v>196</v>
       </c>
       <c r="N204" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O204" s="35">
         <v>1</v>
@@ -28599,7 +28600,7 @@
         <v>190</v>
       </c>
       <c r="I205" s="33" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="J205" s="33">
         <v>99</v>
@@ -28614,7 +28615,7 @@
         <v>196</v>
       </c>
       <c r="N205" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O205" s="35">
         <v>1</v>
@@ -28712,13 +28713,13 @@
         <v>7</v>
       </c>
       <c r="D206" s="34" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="E206" s="34" t="s">
         <v>38</v>
       </c>
       <c r="F206" s="34" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="G206" s="34" t="s">
         <v>72</v>
@@ -28727,7 +28728,7 @@
         <v>190</v>
       </c>
       <c r="I206" s="33" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="J206" s="33">
         <v>4</v>
@@ -28742,7 +28743,7 @@
         <v>196</v>
       </c>
       <c r="N206" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O206" s="35">
         <v>1</v>
@@ -28838,13 +28839,13 @@
         <v>7</v>
       </c>
       <c r="D207" s="34" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="E207" s="34" t="s">
         <v>38</v>
       </c>
       <c r="F207" s="34" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="G207" s="34" t="s">
         <v>88</v>
@@ -28853,7 +28854,7 @@
         <v>190</v>
       </c>
       <c r="I207" s="33" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="J207" s="33">
         <v>2</v>
@@ -28868,7 +28869,7 @@
         <v>196</v>
       </c>
       <c r="N207" s="34" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O207" s="35">
         <v>1</v>
@@ -28970,7 +28971,7 @@
         <v>38</v>
       </c>
       <c r="F208" s="34" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="G208" s="34" t="s">
         <v>82</v>
@@ -28994,7 +28995,7 @@
         <v>196</v>
       </c>
       <c r="N208" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O208" s="35">
         <v>1</v>
@@ -29122,7 +29123,7 @@
         <v>103</v>
       </c>
       <c r="N209" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O209" s="35">
         <v>1</v>
@@ -29494,7 +29495,7 @@
         <v>103</v>
       </c>
       <c r="N212" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O212" s="35">
         <v>1</v>
@@ -29622,7 +29623,7 @@
         <v>103</v>
       </c>
       <c r="N213" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O213" s="35">
         <v>1</v>
@@ -29750,7 +29751,7 @@
         <v>103</v>
       </c>
       <c r="N214" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O214" s="35">
         <v>1</v>
@@ -29851,7 +29852,7 @@
         <v>55</v>
       </c>
       <c r="F215" s="34" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="G215" s="34" t="s">
         <v>145</v>
@@ -29860,7 +29861,7 @@
         <v>190</v>
       </c>
       <c r="I215" s="33" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="J215" s="33">
         <v>99</v>
@@ -29875,7 +29876,7 @@
         <v>103</v>
       </c>
       <c r="N215" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O215" s="35">
         <v>1</v>
@@ -30000,7 +30001,7 @@
         <v>312</v>
       </c>
       <c r="N216" s="37" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="O216" s="38"/>
       <c r="P216" s="36"/>
@@ -30124,7 +30125,7 @@
         <v>196</v>
       </c>
       <c r="N217" s="34" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="O217" s="35">
         <v>1</v>

</xml_diff>

<commit_message>
chore(mappa): aggiornamento automatico 2026-09-03
</commit_message>
<xml_diff>
--- a/Torino_2027.xlsx
+++ b/Torino_2027.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scarg\Dropbox\PNE Simone\Guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA60B790-70E9-4F01-B69B-847B14EF757C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1069DE4B-8219-4A82-9E45-2F99584F873E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="665" xr2:uid="{65E54767-2A5A-433C-9949-276C98563996}"/>
   </bookViews>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2020" uniqueCount="916">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2021" uniqueCount="916">
   <si>
     <t>Recensore</t>
   </si>
@@ -10590,49 +10590,51 @@
       <c r="AT60" s="13"/>
     </row>
     <row r="61" spans="1:46" s="14" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="20">
-        <v>0</v>
-      </c>
-      <c r="B61" s="20">
-        <v>1</v>
-      </c>
-      <c r="C61" s="20">
+      <c r="A61" s="36">
+        <v>0</v>
+      </c>
+      <c r="B61" s="36">
+        <v>1</v>
+      </c>
+      <c r="C61" s="36">
         <v>5</v>
       </c>
-      <c r="D61" s="19" t="s">
+      <c r="D61" s="37" t="s">
         <v>390</v>
       </c>
-      <c r="E61" s="19" t="s">
+      <c r="E61" s="37" t="s">
         <v>237</v>
       </c>
-      <c r="F61" s="19" t="s">
+      <c r="F61" s="37" t="s">
         <v>391</v>
       </c>
-      <c r="G61" s="19" t="s">
+      <c r="G61" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="H61" s="19" t="s">
+      <c r="H61" s="37" t="s">
         <v>190</v>
       </c>
-      <c r="I61" s="20" t="s">
+      <c r="I61" s="36" t="s">
         <v>392</v>
       </c>
-      <c r="J61" s="20">
+      <c r="J61" s="36">
         <v>5</v>
       </c>
-      <c r="K61" s="20" t="s">
+      <c r="K61" s="36" t="s">
         <v>298</v>
       </c>
-      <c r="L61" s="20" t="s">
+      <c r="L61" s="36" t="s">
         <v>305</v>
       </c>
-      <c r="M61" s="19" t="s">
+      <c r="M61" s="37" t="s">
         <v>675</v>
       </c>
-      <c r="N61" s="19"/>
-      <c r="O61" s="18"/>
-      <c r="P61" s="20"/>
-      <c r="Q61" s="19"/>
+      <c r="N61" s="37" t="s">
+        <v>850</v>
+      </c>
+      <c r="O61" s="38"/>
+      <c r="P61" s="36"/>
+      <c r="Q61" s="37"/>
       <c r="R61" s="13"/>
       <c r="S61" s="2">
         <f t="shared" si="23"/>

</xml_diff>